<commit_message>
Update modeling code and generated results
</commit_message>
<xml_diff>
--- a/outputs/result_filled_v2.xlsx
+++ b/outputs/result_filled_v2.xlsx
@@ -423,7 +423,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L22"/>
+  <dimension ref="A1:L26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="13.8"/>
   <cols>
     <col width="15.77734375" customWidth="1" min="4" max="4"/>
@@ -474,7 +474,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>S04</t>
+          <t>S06</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -550,7 +550,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>P03,P04</t>
+          <t>P11</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -590,19 +590,19 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>S01</t>
+          <t>P03,P04</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>射击</t>
+          <t>拍照</t>
         </is>
       </c>
       <c r="D5" t="n">
-        <v>493.75</v>
+        <v>494.05</v>
       </c>
       <c r="E5" t="n">
-        <v>495.25</v>
+        <v>494.55</v>
       </c>
       <c r="H5" s="3" t="n"/>
       <c r="I5" s="3" t="n"/>
@@ -616,19 +616,19 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>S12</t>
+          <t>P10</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>射击</t>
+          <t>拍照</t>
         </is>
       </c>
       <c r="D6" t="n">
-        <v>506.65</v>
+        <v>495.05</v>
       </c>
       <c r="E6" t="n">
-        <v>508.15</v>
+        <v>495.55</v>
       </c>
     </row>
     <row r="7">
@@ -637,7 +637,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>S11</t>
+          <t>S12</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -646,10 +646,10 @@
         </is>
       </c>
       <c r="D7" t="n">
-        <v>508.55</v>
+        <v>506.75</v>
       </c>
       <c r="E7" t="n">
-        <v>510.05</v>
+        <v>508.25</v>
       </c>
     </row>
     <row r="8">
@@ -658,19 +658,19 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>P01,P02</t>
+          <t>S11</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>拍照</t>
+          <t>射击</t>
         </is>
       </c>
       <c r="D8" t="n">
-        <v>510.55</v>
+        <v>508.55</v>
       </c>
       <c r="E8" t="n">
-        <v>511.05</v>
+        <v>510.05</v>
       </c>
     </row>
     <row r="9">
@@ -679,19 +679,19 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>S11</t>
+          <t>P01,P02</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>射击</t>
+          <t>拍照</t>
         </is>
       </c>
       <c r="D9" t="n">
-        <v>512.25</v>
+        <v>510.55</v>
       </c>
       <c r="E9" t="n">
-        <v>513.75</v>
+        <v>511.05</v>
       </c>
     </row>
     <row r="10">
@@ -700,7 +700,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>S10</t>
+          <t>S12</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -709,10 +709,10 @@
         </is>
       </c>
       <c r="D10" t="n">
-        <v>515.15</v>
+        <v>513.75</v>
       </c>
       <c r="E10" t="n">
-        <v>516.65</v>
+        <v>515.25</v>
       </c>
     </row>
     <row r="11">
@@ -721,7 +721,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>S12</t>
+          <t>S11</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -730,10 +730,10 @@
         </is>
       </c>
       <c r="D11" t="n">
+        <v>515.35</v>
+      </c>
+      <c r="E11" t="n">
         <v>516.85</v>
-      </c>
-      <c r="E11" t="n">
-        <v>518.35</v>
       </c>
     </row>
     <row r="12">
@@ -742,7 +742,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>S11</t>
+          <t>S12</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -751,10 +751,10 @@
         </is>
       </c>
       <c r="D12" t="n">
-        <v>522.55</v>
+        <v>516.95</v>
       </c>
       <c r="E12" t="n">
-        <v>524.05</v>
+        <v>518.45</v>
       </c>
     </row>
     <row r="13">
@@ -763,7 +763,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>S10</t>
+          <t>S11</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -772,10 +772,10 @@
         </is>
       </c>
       <c r="D13" t="n">
-        <v>525.25</v>
+        <v>522.15</v>
       </c>
       <c r="E13" t="n">
-        <v>526.75</v>
+        <v>523.65</v>
       </c>
     </row>
     <row r="14">
@@ -784,7 +784,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>S10</t>
+          <t>S11</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -793,10 +793,10 @@
         </is>
       </c>
       <c r="D14" t="n">
-        <v>526.85</v>
+        <v>523.75</v>
       </c>
       <c r="E14" t="n">
-        <v>528.35</v>
+        <v>525.25</v>
       </c>
     </row>
     <row r="15">
@@ -814,10 +814,10 @@
         </is>
       </c>
       <c r="D15" t="n">
-        <v>532.65</v>
+        <v>525.35</v>
       </c>
       <c r="E15" t="n">
-        <v>534.15</v>
+        <v>526.85</v>
       </c>
     </row>
     <row r="16">
@@ -835,10 +835,10 @@
         </is>
       </c>
       <c r="D16" t="n">
-        <v>534.55</v>
+        <v>526.95</v>
       </c>
       <c r="E16" t="n">
-        <v>536.05</v>
+        <v>528.45</v>
       </c>
     </row>
     <row r="17">
@@ -847,7 +847,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>S15</t>
+          <t>S10</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -856,10 +856,10 @@
         </is>
       </c>
       <c r="D17" t="n">
-        <v>748.65</v>
+        <v>531.45</v>
       </c>
       <c r="E17" t="n">
-        <v>750.15</v>
+        <v>532.95</v>
       </c>
     </row>
     <row r="18">
@@ -868,7 +868,7 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>S14</t>
+          <t>S10</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
@@ -877,10 +877,10 @@
         </is>
       </c>
       <c r="D18" t="n">
-        <v>751.45</v>
+        <v>533.15</v>
       </c>
       <c r="E18" t="n">
-        <v>752.95</v>
+        <v>534.65</v>
       </c>
     </row>
     <row r="19">
@@ -889,7 +889,7 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>S13</t>
+          <t>S10</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
@@ -898,10 +898,10 @@
         </is>
       </c>
       <c r="D19" t="n">
-        <v>762.05</v>
+        <v>534.75</v>
       </c>
       <c r="E19" t="n">
-        <v>763.55</v>
+        <v>536.25</v>
       </c>
     </row>
     <row r="20">
@@ -910,7 +910,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>S11</t>
+          <t>S15</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -919,10 +919,10 @@
         </is>
       </c>
       <c r="D20" t="n">
-        <v>763.65</v>
+        <v>748.85</v>
       </c>
       <c r="E20" t="n">
-        <v>765.15</v>
+        <v>750.35</v>
       </c>
     </row>
     <row r="21">
@@ -931,7 +931,7 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>S12</t>
+          <t>S14</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
@@ -940,10 +940,10 @@
         </is>
       </c>
       <c r="D21" t="n">
-        <v>765.25</v>
+        <v>750.45</v>
       </c>
       <c r="E21" t="n">
-        <v>766.75</v>
+        <v>751.95</v>
       </c>
     </row>
     <row r="22">
@@ -952,18 +952,102 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
+          <t>S16</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>射击</t>
+        </is>
+      </c>
+      <c r="D22" t="n">
+        <v>752.05</v>
+      </c>
+      <c r="E22" t="n">
+        <v>753.55</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="n">
+        <v>22</v>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>S13</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>射击</t>
+        </is>
+      </c>
+      <c r="D23" t="n">
+        <v>762.05</v>
+      </c>
+      <c r="E23" t="n">
+        <v>763.55</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="n">
+        <v>23</v>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
           <t>S12</t>
         </is>
       </c>
-      <c r="C22" t="inlineStr">
-        <is>
-          <t>射击</t>
-        </is>
-      </c>
-      <c r="D22" t="n">
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>射击</t>
+        </is>
+      </c>
+      <c r="D24" t="n">
+        <v>763.65</v>
+      </c>
+      <c r="E24" t="n">
+        <v>765.15</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="n">
+        <v>24</v>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>S11</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>射击</t>
+        </is>
+      </c>
+      <c r="D25" t="n">
+        <v>765.55</v>
+      </c>
+      <c r="E25" t="n">
+        <v>767.05</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="n">
+        <v>25</v>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>S12</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>射击</t>
+        </is>
+      </c>
+      <c r="D26" t="n">
         <v>767.45</v>
       </c>
-      <c r="E22" t="n">
+      <c r="E26" t="n">
         <v>768.95</v>
       </c>
     </row>

</xml_diff>